<commit_message>
Add SME chatbot use case (AgentHub) to browser-agent guide; fix contact email transliteration
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DxicrQX4huGPqLPX3WwhZX
</commit_message>
<xml_diff>
--- a/demo-data/Dữ liệu setup/CRM Sale/Bộ dữ liệu demo Synnex FPT (dữ liệu gốc).xlsx
+++ b/demo-data/Dữ liệu setup/CRM Sale/Bộ dữ liệu demo Synnex FPT (dữ liệu gốc).xlsx
@@ -6769,7 +6769,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>đat.pq@saovietmart.vn</t>
+          <t>dat.pq@saovietmart.vn</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -6802,7 +6802,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>phong.đđ@nhatminhtech.vn</t>
+          <t>phong.dd@nhatminhtech.vn</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>huong.đv@nhatminhtech.vn</t>
+          <t>huong.dv@nhatminhtech.vn</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -6872,7 +6872,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>đat.hh@nhatminhtech.vn</t>
+          <t>dat.hh@nhatminhtech.vn</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>ha.đh@phuongdongit.vn</t>
+          <t>ha.dh@phuongdongit.vn</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>nam.đđ@bachkhoahp.vn</t>
+          <t>nam.dd@bachkhoahp.vn</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -7737,7 +7737,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>khoa.hđ@haiaunhatrang.vn</t>
+          <t>khoa.hd@haiaunhatrang.vn</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -7807,7 +7807,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>hung.đh@dongduongdigital.vn</t>
+          <t>hung.dh@dongduongdigital.vn</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>đat.vn@dongduongdigital.vn</t>
+          <t>dat.vn@dongduongdigital.vn</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -7877,7 +7877,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>đat.tt@laptoptaman.vn</t>
+          <t>dat.tt@laptoptaman.vn</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>long.đv@tantientelecom.vn</t>
+          <t>long.dv@tantientelecom.vn</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>thao.đh61@gmail.com</t>
+          <t>thao.dh61@gmail.com</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -8355,7 +8355,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>tuan.đh27@gmail.com</t>
+          <t>tuan.dh27@gmail.com</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -8487,7 +8487,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>linh.đh36@gmail.com</t>
+          <t>linh.dh36@gmail.com</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>đat.nb56@gmail.com</t>
+          <t>dat.nb56@gmail.com</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -8883,7 +8883,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>phong.đh@cds.donghai.gov.vn</t>
+          <t>phong.dh@cds.donghai.gov.vn</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>quan.đn@cds.donghai.gov.vn</t>
+          <t>quan.dn@cds.donghai.gov.vn</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>lan.đm@syt.donghai.gov.vn</t>
+          <t>lan.dm@syt.donghai.gov.vn</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
@@ -9229,7 +9229,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>dung.bđ@hlut.edu.vn</t>
+          <t>dung.bd@hlut.edu.vn</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -9538,7 +9538,7 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>linh.đv@saobaca.bank.vn</t>
+          <t>linh.dv@saobaca.bank.vn</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
@@ -9641,7 +9641,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>ha.lđ@abtinsurance.vn</t>
+          <t>ha.ld@abtinsurance.vn</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>khoa.đm@abtinsurance.vn</t>
+          <t>khoa.dm@abtinsurance.vn</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>đat.bn@saomaitelecom.vn</t>
+          <t>dat.bn@saomaitelecom.vn</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">

</xml_diff>